<commit_message>
Carta Lorena v2: bloque 1 reescrito con la evidencia de sus propias autoevaluaciones (13 sesiones positivas, citas textuales del 15-16-17 sep) en tono respetuoso + invitacion a reunion con expediente; bloques 2 y 3 intactos
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/experiencia_cliente/Lorena/RESPUESTA_LORENA.xlsx
+++ b/recursos/experiencia_cliente/Lorena/RESPUESTA_LORENA.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPUESTA LORENA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPUESTA LORENA v2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -456,129 +456,136 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Tomamos tu comentario con total seriedad. Nuestro programa lleva registro clase a clase (guías de sesión, reportes firmados por el docente y registros de salida de los estudiantes), y coordinación académica está intervieniendo el desarrollo de tu grupo esta misma semana: se están haciendo ajustes concretos. Además queremos decirte algo con la misma franqueza: tu proceso ha funcionado — tus propias autoevaluaciones muestran tu avance desde que empezaste, y tú misma nos escribiste que al principio el curso te sirvió mucho. Has aprendido, y con los ajustes en marcha vas a seguir aprendiendo. Por eso, antes de cualquier decisión, te invitamos a una reunión presencial esta semana y a darle a tu grupo las próximas dos semanas con los cambios andando.</t>
+          <t>Tomamos tu comentario con total seriedad, y por eso lo primero que hizo coordinación fue revisar el registro completo de tu grupo — y tu propio expediente. Queremos compartirte lo que encontramos, con respeto y con datos: tus autoevaluaciones, diligenciadas por ti clase a clase, registran trece sesiones consecutivas calificadas positivamente, con el contenido académico de cada día anotado por ti misma — condicionales, presente perfecto, phrasal verbs, voz pasiva. Incluso el 15 de septiembre, el mismo día de tus correos, tu registro de clase dice "Bien, aprendimos sobre preguntar precios"; el 16, "practicamos bastante speaking"; y el 17, "hablamos bastante y escuchamos audios".</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Eso no le resta valor a tu inconformidad — le da contexto: lo que tu expediente muestra no es un curso que dejó de funcionar, sino una estudiante que ha avanzado de verdad y que llegó a la parte del camino donde el avance se siente menos y cuesta más. Eso pasa exactamente al final del A2 y en B1, y es la etapa que separa a los que llegan de los que casi llegan. Tú has demostrado ser de las que llegan — sería una lástima que te lo quitaras a ti misma justo aquí. Te invitamos a una reunión presencial esta semana para conversarlo mirando tu expediente juntas.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>2. EL ESTADO DE TU CONTRATO, COMO LO SOLICITAS</t>
-        </is>
-      </c>
+      <c r="A8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Tu contrato No. 2437 del 2 de julio de 2026 corresponde al programa completo A1→B2 por $5.099.144 — un PRECIO DE PAQUETE con un beneficio condicionado a completar el programa: el mismo programa a tarifa plena vale $8.696.000, y las cláusulas 8, 16 y 17 que leíste e inicialaste una a una establecen que el paquete no contempla congelaciones, devoluciones ni terminaciones parciales, y que quien no esté seguro de continuar debe optar por niveles individuales.</t>
+          <t>2. EL ESTADO DE TU CONTRATO, COMO LO SOLICITAS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Valores pagados a la fecha: $3.033.048 (abono de $2.000.000 y dos cuotas de $516.524).</t>
+          <t>Tu contrato No. 2437 del 2 de julio de 2026 corresponde al programa completo A1→B2 por $5.099.144 — un PRECIO DE PAQUETE con un beneficio condicionado a completar el programa: el mismo programa a tarifa plena vale $8.696.000, y las cláusulas 8, 16 y 17 que leíste e inicialaste una a una establecen que el paquete no contempla congelaciones, devoluciones ni terminaciones parciales, y que quien no esté seguro de continuar debe optar por niveles individuales.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
+          <t>Valores pagados a la fecha: $3.033.048 (abono de $2.000.000 y dos cuotas de $516.524).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
           <t>Obligación vigente conforme al contrato y al pagaré suscrito: $2.066.096 (cuatro cuotas restantes).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>3. NUESTRA ALTERNATIVA DE CIERRE — POR ÚNICA VEZ</t>
-        </is>
-      </c>
+      <c r="A13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>No obstante lo anterior, y valorando tu proceso con nosotros, si tu decisión final es retirarte al culminar tu nivel A2, te ofrecemos esta alternativa: liquidar únicamente lo efectivamente cursado, a la tarifa individual vigente de cada nivel, así:</t>
+          <t>3. NUESTRA ALTERNATIVA DE CIERRE — POR ÚNICA VEZ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>· Nivel A1 (cursado): $1.596.000</t>
+          <t>No obstante lo anterior, y valorando tu proceso con nosotros, si tu decisión final es retirarte al culminar tu nivel A2, te ofrecemos esta alternativa: liquidar únicamente lo efectivamente cursado, a la tarifa individual vigente de cada nivel, así:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>· Nivel A2 (en curso, a culminar): $1.915.000</t>
+          <t>· Nivel A1 (cursado): $1.596.000</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>· Total servicios a tarifa individual: $3.511.000</t>
+          <t>· Nivel A2 (en curso, a culminar): $1.915.000</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>· Total pagado por ti: $3.033.048</t>
+          <t>· Total servicios a tarifa individual: $3.511.000</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>· SALDO A TU CARGO CON ESTA ALTERNATIVA: $477.952</t>
+          <t>· Total pagado por ti: $3.033.048</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Pagando ese saldo, firmamos Acta de Paz y Salvo: tu pagaré se anula y se te devuelve, no queda ninguna obligación entre las partes, y recibes tus certificados oficiales de los niveles cursados y aprobados.</t>
+          <t>· SALDO A TU CARGO CON ESTA ALTERNATIVA: $477.952</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
+          <t>Pagando ese saldo, firmamos Acta de Paz y Salvo: tu pagaré se anula y se te devuelve, no queda ninguna obligación entre las partes, y recibes tus certificados oficiales de los niveles cursados y aprobados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
           <t>Esta alternativa está disponible hasta el 30 de septiembre de 2026. Después de esa fecha, aplican los términos ordinarios del contrato y del pagaré.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr"/>
-    </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="A23" s="1" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Quedamos atentos a coordinar la reunión de esta semana — nos gustaría mucho más verte terminar tu programa que firmarte un paz y salvo.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>Cordialmente,</t>
-        </is>
-      </c>
+      <c r="A25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>Cordialmente,</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Depto. Experiencia al Cliente — Heiiu English Academy</t>
         </is>

</xml_diff>

<commit_message>
Carta Lorena: salida de 477.952 sale del correo a hoja 'PARA LA REUNION - NO ENVIAR'; el correo cierra anunciando alternativas de cierre en la reunion sin dar el numero
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/recursos/experiencia_cliente/Lorena/RESPUESTA_LORENA.xlsx
+++ b/recursos/experiencia_cliente/Lorena/RESPUESTA_LORENA.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RESPUESTA LORENA v2" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARA LA REUNION - NO ENVIAR" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,7 +435,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr"/>
+      <c r="A2" s="1" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -444,7 +445,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr"/>
+      <c r="A4" s="1" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -468,7 +469,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr"/>
+      <c r="A8" s="1" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -499,95 +500,149 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr"/>
+      <c r="A13" s="1" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>3. NUESTRA ALTERNATIVA DE CIERRE — POR ÚNICA VEZ</t>
+          <t>Si después de conversarlo tu decisión sigue siendo retirarte, en esa misma reunión revisamos contigo las alternativas de cierre que contempla tu contrato. Te proponemos reunirnos esta semana en la sede, en el horario que te sirva — quedamos atentos a tu respuesta. Nos gustaría mucho más verte terminar tu programa que firmarte un paz y salvo.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>No obstante lo anterior, y valorando tu proceso con nosotros, si tu decisión final es retirarte al culminar tu nivel A2, te ofrecemos esta alternativa: liquidar únicamente lo efectivamente cursado, a la tarifa individual vigente de cada nivel, así:</t>
-        </is>
-      </c>
+      <c r="A15" s="1" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>· Nivel A1 (cursado): $1.596.000</t>
+          <t>Cordialmente,</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
+          <t>Depto. Experiencia al Cliente — Heiiu English Academy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SOLO PARA LA REUNIÓN. Se ofrece únicamente si Lorena insiste en retirarse. Después de ofrecerla, dejarla por escrito en un correo de seguimiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>3. NUESTRA ALTERNATIVA DE CIERRE — POR ÚNICA VEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No obstante lo anterior, y valorando tu proceso con nosotros, si tu decisión final es retirarte al culminar tu nivel A2, te ofrecemos esta alternativa: liquidar únicamente lo efectivamente cursado, a la tarifa individual vigente de cada nivel, así:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>· Nivel A1 (cursado): $1.596.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
           <t>· Nivel A2 (en curso, a culminar): $1.915.000</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>· Total servicios a tarifa individual: $3.511.000</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>· Total pagado por ti: $3.033.048</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>· SALDO A TU CARGO CON ESTA ALTERNATIVA: $477.952</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Pagando ese saldo, firmamos Acta de Paz y Salvo: tu pagaré se anula y se te devuelve, no queda ninguna obligación entre las partes, y recibes tus certificados oficiales de los niveles cursados y aprobados.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Esta alternativa está disponible hasta el 30 de septiembre de 2026. Después de esa fecha, aplican los términos ordinarios del contrato y del pagaré.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>Quedamos atentos a coordinar la reunión de esta semana — nos gustaría mucho más verte terminar tu programa que firmarte un paz y salvo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>Cordialmente,</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Depto. Experiencia al Cliente — Heiiu English Academy</t>
         </is>
       </c>
     </row>

</xml_diff>